<commit_message>
Label lesson action buttons Continue and import that label from the workbook.
The Instructions sheet now has a button field so each section can set the word learners see.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/inroads-mvp-import-template/lesson.xlsx
+++ b/public/inroads-mvp-import-template/lesson.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="773" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="782" uniqueCount="142">
   <si>
     <t>key</t>
   </si>
@@ -76,6 +76,12 @@
   </si>
   <si>
     <t>Observe Challenge</t>
+  </si>
+  <si>
+    <t>button</t>
+  </si>
+  <si>
+    <t>Continue</t>
   </si>
   <si>
     <t>second_instruction</t>
@@ -478,12 +484,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -887,7 +894,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -929,10 +936,10 @@
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="A4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="3" t="s">
         <v>20</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -1117,10 +1124,10 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>15</v>
+      </c>
+      <c r="B21" t="s">
         <v>54</v>
-      </c>
-      <c r="B21" t="s">
-        <v>16</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>55</v>
@@ -1128,76 +1135,76 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B22" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B23" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B24" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C23" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>54</v>
-      </c>
-      <c r="B24" t="s">
-        <v>52</v>
-      </c>
       <c r="C24" s="2" t="s">
-        <v>58</v>
+        <v>21</v>
       </c>
     </row>
     <row r="25" hidden="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B25" t="s">
+        <v>22</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="C25" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="B26" t="s">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>56</v>
+      </c>
+      <c r="B27" t="s">
         <v>61</v>
       </c>
-      <c r="B27" t="s">
-        <v>18</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>63</v>
+      <c r="C27" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B28" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>64</v>
@@ -1205,24 +1212,57 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B29" t="s">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="30" hidden="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+      <c r="A30" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>63</v>
+      </c>
+      <c r="B31" t="s">
+        <v>22</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>63</v>
+      </c>
+      <c r="B32" t="s">
+        <v>54</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>63</v>
+      </c>
+      <c r="B33" t="s">
         <v>61</v>
       </c>
-      <c r="B30" t="s">
-        <v>59</v>
-      </c>
-      <c r="C30" t="s">
-        <v>60</v>
+      <c r="C33" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -1234,7 +1274,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:U31"/>
+  <dimension ref="A1:T31"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -1252,69 +1292,69 @@
     <col min="14" max="20" width="10" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>15</v>
       </c>
@@ -1322,37 +1362,37 @@
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="J2">
         <v>10</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="L2">
         <v>0</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="N2">
         <v>0</v>
@@ -1376,45 +1416,45 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="L3">
         <v>10</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="N3">
         <v>0</v>
@@ -1438,45 +1478,45 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="J4">
         <v>10</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="L4">
         <v>0</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="N4">
         <v>0</v>
@@ -1500,45 +1540,45 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="L5">
         <v>10</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="N5">
         <v>0</v>
@@ -1562,45 +1602,45 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B6">
         <v>2</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="J6">
         <v>10</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="L6">
         <v>0</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="N6">
         <v>0</v>
@@ -1624,45 +1664,45 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="J7">
         <v>10</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="L7">
         <v>0</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="N7">
         <v>0</v>
@@ -1686,45 +1726,45 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B8">
         <v>1</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="J8">
         <v>10</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="L8">
         <v>0</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="N8">
         <v>0</v>
@@ -1748,45 +1788,45 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="J9">
         <v>0</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="L9">
         <v>10</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="N9">
         <v>0</v>
@@ -1810,45 +1850,45 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B10">
         <v>2</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="J10">
         <v>10</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="L10">
         <v>0</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="N10">
         <v>0</v>
@@ -1872,7 +1912,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>5</v>
       </c>
@@ -1934,7 +1974,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>5</v>
       </c>
@@ -1996,7 +2036,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>5</v>
       </c>
@@ -2058,7 +2098,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>5</v>
       </c>
@@ -2120,7 +2160,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>5</v>
       </c>
@@ -2182,7 +2222,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>5</v>
       </c>
@@ -2244,7 +2284,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>5</v>
       </c>
@@ -2306,7 +2346,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>5</v>
       </c>
@@ -2368,7 +2408,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>5</v>
       </c>
@@ -2430,7 +2470,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>5</v>
       </c>
@@ -2492,7 +2532,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>5</v>
       </c>
@@ -2554,7 +2594,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>5</v>
       </c>
@@ -2616,7 +2656,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>5</v>
       </c>
@@ -2678,7 +2718,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>5</v>
       </c>
@@ -2740,7 +2780,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>5</v>
       </c>
@@ -2802,7 +2842,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>5</v>
       </c>
@@ -2864,7 +2904,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>5</v>
       </c>
@@ -2926,7 +2966,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>5</v>
       </c>
@@ -2988,7 +3028,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>5</v>
       </c>
@@ -3050,7 +3090,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>5</v>
       </c>
@@ -3112,7 +3152,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>5</v>
       </c>
@@ -3201,21 +3241,21 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>9</v>
@@ -3223,32 +3263,32 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>9</v>
@@ -3256,10 +3296,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>11</v>
@@ -3267,32 +3307,32 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>134</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>130</v>
-      </c>
       <c r="C7" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>9</v>
@@ -3300,10 +3340,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>11</v>
@@ -3311,32 +3351,32 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>9</v>
@@ -3344,10 +3384,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>137</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>135</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>133</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>11</v>
@@ -3355,32 +3395,32 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>9</v>
@@ -3388,10 +3428,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>11</v>
@@ -3399,32 +3439,32 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>9</v>
@@ -3432,10 +3472,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>11</v>
@@ -3443,32 +3483,32 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>9</v>
@@ -3476,32 +3516,32 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>9</v>
@@ -3509,10 +3549,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>11</v>

</xml_diff>

<commit_message>
Read lesson button text and the title description from the workbook.
One Lesson sheet cell labels every Continue button, and the title card shows the lesson description.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/inroads-mvp-import-template/lesson.xlsx
+++ b/public/inroads-mvp-import-template/lesson.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="782" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="142">
   <si>
     <t>key</t>
   </si>
@@ -50,6 +50,12 @@
   </si>
   <si>
     <t>English</t>
+  </si>
+  <si>
+    <t>button</t>
+  </si>
+  <si>
+    <t>Continue</t>
   </si>
   <si>
     <t>section</t>
@@ -76,12 +82,6 @@
   </si>
   <si>
     <t>Observe Challenge</t>
-  </si>
-  <si>
-    <t>button</t>
-  </si>
-  <si>
-    <t>Continue</t>
   </si>
   <si>
     <t>second_instruction</t>
@@ -830,7 +830,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -885,6 +885,14 @@
         <v>11</v>
       </c>
     </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection sheet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -894,7 +902,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -904,233 +912,233 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>20</v>
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" t="s">
+        <v>22</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B9" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B12" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B15" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B16" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B17" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B20" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>15</v>
+        <v>56</v>
       </c>
       <c r="B21" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -1138,10 +1146,10 @@
         <v>56</v>
       </c>
       <c r="B22" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -1149,54 +1157,54 @@
         <v>56</v>
       </c>
       <c r="B23" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
+      <c r="A24" t="s">
         <v>56</v>
       </c>
-      <c r="B24" s="3" t="s">
-        <v>20</v>
+      <c r="B24" t="s">
+        <v>54</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="25" hidden="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>56</v>
       </c>
       <c r="B25" t="s">
-        <v>22</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
+      </c>
+      <c r="C25" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="B26" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="B27" t="s">
-        <v>61</v>
-      </c>
-      <c r="C27" t="s">
-        <v>62</v>
+        <v>20</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -1204,10 +1212,10 @@
         <v>63</v>
       </c>
       <c r="B28" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -1215,53 +1223,20 @@
         <v>63</v>
       </c>
       <c r="B29" t="s">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="30" hidden="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>63</v>
       </c>
-      <c r="B30" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>63</v>
-      </c>
-      <c r="B31" t="s">
-        <v>22</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>63</v>
-      </c>
-      <c r="B32" t="s">
-        <v>54</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>63</v>
-      </c>
-      <c r="B33" t="s">
+      <c r="B30" t="s">
         <v>61</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C30" t="s">
         <v>62</v>
       </c>
     </row>
@@ -1294,7 +1269,7 @@
   <sheetData>
     <row r="1" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>68</v>
@@ -1356,7 +1331,7 @@
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B2">
         <v>1</v>

</xml_diff>

<commit_message>
Read the severity Submit label and title-card country from the lesson workbook.
Severity questions use the Lesson sheet submit cell, and the title card shows the lesson country.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/inroads-mvp-import-template/lesson.xlsx
+++ b/public/inroads-mvp-import-template/lesson.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="777" uniqueCount="144">
   <si>
     <t>key</t>
   </si>
@@ -56,6 +56,12 @@
   </si>
   <si>
     <t>Continue</t>
+  </si>
+  <si>
+    <t>submit</t>
+  </si>
+  <si>
+    <t>Submit</t>
   </si>
   <si>
     <t>section</t>
@@ -484,13 +490,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -830,7 +835,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -886,11 +891,19 @@
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+      <c r="A7" t="s">
         <v>12</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -912,332 +925,332 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B12" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B13" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B16" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B17" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B18" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B19" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B21" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B22" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B23" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>58</v>
+      </c>
+      <c r="B24" t="s">
         <v>56</v>
       </c>
-      <c r="B24" t="s">
-        <v>54</v>
-      </c>
       <c r="C24" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B25" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C25" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B26" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B27" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B28" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B29" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>65</v>
+      </c>
+      <c r="B30" t="s">
         <v>63</v>
       </c>
-      <c r="B30" t="s">
-        <v>61</v>
-      </c>
       <c r="C30" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -1269,105 +1282,105 @@
   <sheetData>
     <row r="1" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="J2">
         <v>10</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="L2">
         <v>0</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="N2">
         <v>0</v>
@@ -1393,43 +1406,43 @@
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="L3">
         <v>10</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="N3">
         <v>0</v>
@@ -1455,43 +1468,43 @@
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="J4">
         <v>10</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="L4">
         <v>0</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="N4">
         <v>0</v>
@@ -1517,43 +1530,43 @@
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L5">
         <v>10</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="N5">
         <v>0</v>
@@ -1579,43 +1592,43 @@
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B6">
         <v>2</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="J6">
         <v>10</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="L6">
         <v>0</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="N6">
         <v>0</v>
@@ -1641,43 +1654,43 @@
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="J7">
         <v>10</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="L7">
         <v>0</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="N7">
         <v>0</v>
@@ -1703,43 +1716,43 @@
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B8">
         <v>1</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J8">
         <v>10</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="L8">
         <v>0</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="N8">
         <v>0</v>
@@ -1765,43 +1778,43 @@
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="J9">
         <v>0</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="L9">
         <v>10</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="N9">
         <v>0</v>
@@ -1827,43 +1840,43 @@
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B10">
         <v>2</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="J10">
         <v>10</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="L10">
         <v>0</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="N10">
         <v>0</v>
@@ -3216,21 +3229,21 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>9</v>
@@ -3238,32 +3251,32 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>9</v>
@@ -3271,10 +3284,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>11</v>
@@ -3282,32 +3295,32 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>136</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>132</v>
-      </c>
       <c r="C7" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>9</v>
@@ -3315,10 +3328,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>11</v>
@@ -3326,32 +3339,32 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>9</v>
@@ -3359,10 +3372,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>139</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>137</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>135</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>11</v>
@@ -3370,32 +3383,32 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>9</v>
@@ -3403,10 +3416,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>11</v>
@@ -3414,32 +3427,32 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>9</v>
@@ -3447,10 +3460,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>11</v>
@@ -3458,32 +3471,32 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>9</v>
@@ -3491,32 +3504,32 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>9</v>
@@ -3524,10 +3537,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>11</v>

</xml_diff>

<commit_message>
Read the final results headings from the lesson workbook.
Challenge Complete and Challenge Failed come from Lesson sheet cells so each lesson can set that copy.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/inroads-mvp-import-template/lesson.xlsx
+++ b/public/inroads-mvp-import-template/lesson.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="777" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="781" uniqueCount="148">
   <si>
     <t>key</t>
   </si>
@@ -62,6 +62,18 @@
   </si>
   <si>
     <t>Submit</t>
+  </si>
+  <si>
+    <t>challenge_passed</t>
+  </si>
+  <si>
+    <t>Challenge Complete</t>
+  </si>
+  <si>
+    <t>challenge_failed</t>
+  </si>
+  <si>
+    <t>Challenge Failed</t>
   </si>
   <si>
     <t>section</t>
@@ -835,7 +847,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -904,6 +916,22 @@
       </c>
       <c r="B8" s="2" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -925,332 +953,332 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B8" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B9" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B10" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B14" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B15" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B16" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B17" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B18" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B19" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B20" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B21" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B22" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B23" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B24" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B25" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C25" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B26" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B27" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B28" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B29" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B30" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C30" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -1282,105 +1310,105 @@
   <sheetData>
     <row r="1" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="J2">
         <v>10</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="L2">
         <v>0</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="N2">
         <v>0</v>
@@ -1406,43 +1434,43 @@
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="L3">
         <v>10</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="N3">
         <v>0</v>
@@ -1468,43 +1496,43 @@
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="J4">
         <v>10</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="L4">
         <v>0</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="N4">
         <v>0</v>
@@ -1530,43 +1558,43 @@
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="L5">
         <v>10</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="N5">
         <v>0</v>
@@ -1592,43 +1620,43 @@
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B6">
         <v>2</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="J6">
         <v>10</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="L6">
         <v>0</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="N6">
         <v>0</v>
@@ -1654,43 +1682,43 @@
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="J7">
         <v>10</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="L7">
         <v>0</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="N7">
         <v>0</v>
@@ -1716,43 +1744,43 @@
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B8">
         <v>1</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="J8">
         <v>10</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="L8">
         <v>0</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="N8">
         <v>0</v>
@@ -1778,43 +1806,43 @@
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="J9">
         <v>0</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="L9">
         <v>10</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="N9">
         <v>0</v>
@@ -1840,43 +1868,43 @@
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B10">
         <v>2</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="J10">
         <v>10</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="L10">
         <v>0</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="N10">
         <v>0</v>
@@ -3229,21 +3257,21 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>9</v>
@@ -3251,32 +3279,32 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>9</v>
@@ -3284,10 +3312,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>11</v>
@@ -3295,32 +3323,32 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>9</v>
@@ -3328,10 +3356,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>11</v>
@@ -3339,32 +3367,32 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>142</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>134</v>
-      </c>
       <c r="C11" s="2" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>9</v>
@@ -3372,10 +3400,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>11</v>
@@ -3383,32 +3411,32 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>143</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>139</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>9</v>
@@ -3416,10 +3444,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>11</v>
@@ -3427,32 +3455,32 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>9</v>
@@ -3460,10 +3488,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>145</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>141</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>137</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>11</v>
@@ -3471,32 +3499,32 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>9</v>
@@ -3504,32 +3532,32 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>9</v>
@@ -3537,10 +3565,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>11</v>

</xml_diff>

<commit_message>
Read the Observe clip-intro headings from the lesson workbook.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/inroads-mvp-import-template/lesson.xlsx
+++ b/public/inroads-mvp-import-template/lesson.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="781" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="791" uniqueCount="153">
   <si>
     <t>key</t>
   </si>
@@ -74,6 +74,21 @@
   </si>
   <si>
     <t>Challenge Failed</t>
+  </si>
+  <si>
+    <t>Maneuver</t>
+  </si>
+  <si>
+    <t>Roadway</t>
+  </si>
+  <si>
+    <t>Traffic Density</t>
+  </si>
+  <si>
+    <t>Time of Day</t>
+  </si>
+  <si>
+    <t>Road Conditions</t>
   </si>
   <si>
     <t>section</t>
@@ -847,7 +862,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -932,6 +947,46 @@
       </c>
       <c r="B10" s="2" t="s">
         <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -953,332 +1008,332 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B5" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B6" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B7" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B9" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B10" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B11" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B12" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B13" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B14" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B15" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B16" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B17" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B18" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B19" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B20" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="B21" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="B22" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="B23" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="B24" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="B25" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C25" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B26" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B27" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B28" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B29" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B30" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C30" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1310,105 +1365,105 @@
   <sheetData>
     <row r="1" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="J2">
         <v>10</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="L2">
         <v>0</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="N2">
         <v>0</v>
@@ -1434,43 +1489,43 @@
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="L3">
         <v>10</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="N3">
         <v>0</v>
@@ -1496,43 +1551,43 @@
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>103</v>
-      </c>
       <c r="H4" s="2" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="J4">
         <v>10</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="L4">
         <v>0</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="N4">
         <v>0</v>
@@ -1558,43 +1613,43 @@
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="L5">
         <v>10</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="N5">
         <v>0</v>
@@ -1620,43 +1675,43 @@
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="B6">
         <v>2</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="J6">
         <v>10</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="L6">
         <v>0</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="N6">
         <v>0</v>
@@ -1682,43 +1737,43 @@
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="J7">
         <v>10</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="L7">
         <v>0</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="N7">
         <v>0</v>
@@ -1744,43 +1799,43 @@
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B8">
         <v>1</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="J8">
         <v>10</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="L8">
         <v>0</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="N8">
         <v>0</v>
@@ -1806,43 +1861,43 @@
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="J9">
         <v>0</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="L9">
         <v>10</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="N9">
         <v>0</v>
@@ -1868,43 +1923,43 @@
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B10">
         <v>2</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="J10">
         <v>10</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="L10">
         <v>0</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="N10">
         <v>0</v>
@@ -3257,21 +3312,21 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>9</v>
@@ -3279,32 +3334,32 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>9</v>
@@ -3312,10 +3367,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>11</v>
@@ -3323,32 +3378,32 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>147</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>142</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>137</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>9</v>
@@ -3356,10 +3411,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>11</v>
@@ -3367,32 +3422,32 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>9</v>
@@ -3400,10 +3455,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>11</v>
@@ -3411,32 +3466,32 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>148</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>138</v>
-      </c>
       <c r="C15" s="2" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>9</v>
@@ -3444,10 +3499,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>11</v>
@@ -3455,32 +3510,32 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>149</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>144</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>9</v>
@@ -3488,10 +3543,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>11</v>
@@ -3499,32 +3554,32 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>9</v>
@@ -3532,32 +3587,32 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>9</v>
@@ -3565,10 +3620,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>11</v>

</xml_diff>

<commit_message>
Read the final results labels from the lesson workbook.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/inroads-mvp-import-template/lesson.xlsx
+++ b/public/inroads-mvp-import-template/lesson.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="791" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="813" uniqueCount="163">
   <si>
     <t>key</t>
   </si>
@@ -89,6 +89,39 @@
   </si>
   <si>
     <t>Road Conditions</t>
+  </si>
+  <si>
+    <t>pts</t>
+  </si>
+  <si>
+    <t>Detection</t>
+  </si>
+  <si>
+    <t>Accuracy</t>
+  </si>
+  <si>
+    <t>Coaching</t>
+  </si>
+  <si>
+    <t>Q1</t>
+  </si>
+  <si>
+    <t>Q2</t>
+  </si>
+  <si>
+    <t>Q3</t>
+  </si>
+  <si>
+    <t>Q4</t>
+  </si>
+  <si>
+    <t>Observation</t>
+  </si>
+  <si>
+    <t>Process</t>
+  </si>
+  <si>
+    <t>Anticipation</t>
   </si>
   <si>
     <t>section</t>
@@ -225,9 +258,6 @@
     <t xml:space="preserve">You're about to watch a short driving video one time with no replay or side-to-side scanning options. 
 Assess what's happening, what's changing, and why it matters in the scenario. 
 Right after, you'll answer three quick questions about what you saw. You'll get feedback after each question.</t>
-  </si>
-  <si>
-    <t>Process</t>
   </si>
   <si>
     <t xml:space="preserve">Let's look at a couple of points that can strengthen your Process skills. </t>
@@ -862,7 +892,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -987,6 +1017,94 @@
       </c>
       <c r="B15" s="2" t="s">
         <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>28</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>29</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>30</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>31</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>32</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>33</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>34</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>35</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1008,332 +1126,332 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B2" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B3" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B13" t="s">
-        <v>51</v>
+        <v>62</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B14" t="s">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B15" t="s">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B16" t="s">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B17" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>62</v>
+        <v>73</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B20" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="B21" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="B22" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>69</v>
+        <v>34</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="B23" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="B24" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="B25" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="C25" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="B26" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="B27" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="B28" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="B29" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="B30" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="C30" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -1365,105 +1483,105 @@
   <sheetData>
     <row r="1" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="J2">
         <v>10</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="L2">
         <v>0</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="N2">
         <v>0</v>
@@ -1489,43 +1607,43 @@
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="L3">
         <v>10</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="N3">
         <v>0</v>
@@ -1551,43 +1669,43 @@
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="J4">
         <v>10</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="L4">
         <v>0</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="N4">
         <v>0</v>
@@ -1613,43 +1731,43 @@
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="D5" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>109</v>
-      </c>
       <c r="I5" s="2" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="L5">
         <v>10</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>122</v>
+        <v>132</v>
       </c>
       <c r="N5">
         <v>0</v>
@@ -1675,43 +1793,43 @@
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="B6">
         <v>2</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="J6">
         <v>10</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="L6">
         <v>0</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="N6">
         <v>0</v>
@@ -1737,43 +1855,43 @@
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="J7">
         <v>10</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="L7">
         <v>0</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="N7">
         <v>0</v>
@@ -1799,43 +1917,43 @@
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="B8">
         <v>1</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="J8">
         <v>10</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
       <c r="L8">
         <v>0</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
       <c r="N8">
         <v>0</v>
@@ -1861,43 +1979,43 @@
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>133</v>
+        <v>143</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="J9">
         <v>0</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="L9">
         <v>10</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="N9">
         <v>0</v>
@@ -1923,43 +2041,43 @@
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="B10">
         <v>2</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="J10">
         <v>10</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="L10">
         <v>0</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="N10">
         <v>0</v>
@@ -3312,21 +3430,21 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>140</v>
+        <v>150</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>9</v>
@@ -3334,32 +3452,32 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>143</v>
+        <v>153</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>144</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>9</v>
@@ -3367,10 +3485,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>11</v>
@@ -3378,32 +3496,32 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>143</v>
+        <v>153</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>144</v>
+        <v>154</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>147</v>
+        <v>157</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>9</v>
@@ -3411,10 +3529,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>147</v>
+        <v>157</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>11</v>
@@ -3422,32 +3540,32 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>147</v>
+        <v>157</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>143</v>
+        <v>153</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>144</v>
+        <v>154</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>147</v>
+        <v>157</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>9</v>
@@ -3455,10 +3573,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>11</v>
@@ -3466,32 +3584,32 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>143</v>
+        <v>153</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>144</v>
+        <v>154</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>149</v>
+        <v>159</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>9</v>
@@ -3499,10 +3617,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>149</v>
+        <v>159</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>11</v>
@@ -3510,32 +3628,32 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>149</v>
+        <v>159</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>143</v>
+        <v>153</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>144</v>
+        <v>154</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>149</v>
+        <v>159</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>150</v>
+        <v>160</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>9</v>
@@ -3543,10 +3661,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>150</v>
+        <v>160</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>11</v>
@@ -3554,32 +3672,32 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>150</v>
+        <v>160</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>143</v>
+        <v>153</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>144</v>
+        <v>154</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>150</v>
+        <v>160</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>151</v>
+        <v>161</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>9</v>
@@ -3587,32 +3705,32 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>151</v>
+        <v>161</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>143</v>
+        <v>153</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>144</v>
+        <v>154</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>151</v>
+        <v>161</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>162</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>152</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>142</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>9</v>
@@ -3620,10 +3738,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>152</v>
+        <v>162</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>11</v>

</xml_diff>

<commit_message>
Add a SKU field to the Inroads MVP lesson and workbook.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/inroads-mvp-import-template/lesson.xlsx
+++ b/public/inroads-mvp-import-template/lesson.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="813" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="815" uniqueCount="164">
   <si>
     <t>key</t>
   </si>
@@ -32,6 +32,9 @@
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <t>sku</t>
   </si>
   <si>
     <t>intro_first_visit</t>
@@ -547,12 +550,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -892,7 +896,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -923,65 +927,65 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" hidden="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" hidden="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="B5" t="s">
         <v>8</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>12</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>14</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>16</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>18</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>20</v>
@@ -1105,6 +1109,14 @@
       </c>
       <c r="B26" s="2" t="s">
         <v>35</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>36</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -1126,332 +1138,332 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B11" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B13" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B14" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B15" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B16" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B17" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B19" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B20" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B21" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B22" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B23" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B24" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B25" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C25" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B26" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B27" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B28" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B29" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>85</v>
+      </c>
+      <c r="B30" t="s">
+        <v>83</v>
+      </c>
+      <c r="C30" t="s">
         <v>84</v>
-      </c>
-      <c r="B30" t="s">
-        <v>82</v>
-      </c>
-      <c r="C30" t="s">
-        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -1483,105 +1495,105 @@
   <sheetData>
     <row r="1" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J2">
         <v>10</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="L2">
         <v>0</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="N2">
         <v>0</v>
@@ -1607,43 +1619,43 @@
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="L3">
         <v>10</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N3">
         <v>0</v>
@@ -1669,43 +1681,43 @@
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J4">
         <v>10</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="L4">
         <v>0</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="N4">
         <v>0</v>
@@ -1731,43 +1743,43 @@
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="L5">
         <v>10</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="N5">
         <v>0</v>
@@ -1793,43 +1805,43 @@
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B6">
         <v>2</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J6">
         <v>10</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="L6">
         <v>0</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="N6">
         <v>0</v>
@@ -1855,43 +1867,43 @@
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D7" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>134</v>
-      </c>
       <c r="F7" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J7">
         <v>10</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L7">
         <v>0</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="N7">
         <v>0</v>
@@ -1917,43 +1929,43 @@
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B8">
         <v>1</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="J8">
         <v>10</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L8">
         <v>0</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="N8">
         <v>0</v>
@@ -1979,43 +1991,43 @@
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J9">
         <v>0</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="L9">
         <v>10</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="N9">
         <v>0</v>
@@ -2041,43 +2053,43 @@
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B10">
         <v>2</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J10">
         <v>10</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="L10">
         <v>0</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="N10">
         <v>0</v>
@@ -3430,321 +3442,321 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>156</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>155</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>158</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>156</v>
-      </c>
       <c r="C10" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Export the open lesson as a workbook template and refine language versioning.
Download template fills from the version on screen without media, country is set on create and shared across languages, and the editor chrome for switching versions is tightened.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/inroads-mvp-import-template/lesson.xlsx
+++ b/public/inroads-mvp-import-template/lesson.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="815" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="813" uniqueCount="163">
   <si>
     <t>key</t>
   </si>
@@ -41,12 +41,6 @@
   </si>
   <si>
     <t>false</t>
-  </si>
-  <si>
-    <t>country</t>
-  </si>
-  <si>
-    <t>Canada</t>
   </si>
   <si>
     <t>language</t>
@@ -482,6 +476,9 @@
   </si>
   <si>
     <t>Country</t>
+  </si>
+  <si>
+    <t>Canada</t>
   </si>
   <si>
     <t>Vehicle Type</t>
@@ -550,13 +547,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -896,7 +892,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -928,7 +924,7 @@
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" t="s">
         <v>6</v>
       </c>
       <c r="B4" s="2" t="s">
@@ -988,135 +984,127 @@
         <v>19</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>36</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -1138,332 +1126,332 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>40</v>
-      </c>
-      <c r="B2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B7" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B8" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B9" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B12" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B13" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B14" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B15" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B17" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B18" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B19" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B20" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B21" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B22" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>77</v>
+      </c>
+      <c r="B23" t="s">
+        <v>43</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>79</v>
-      </c>
-      <c r="B23" t="s">
-        <v>45</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B24" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B25" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C25" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B26" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>83</v>
+      </c>
+      <c r="B27" t="s">
+        <v>41</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>85</v>
-      </c>
-      <c r="B27" t="s">
-        <v>43</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B28" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B29" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B30" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C30" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -1495,105 +1483,105 @@
   <sheetData>
     <row r="1" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>112</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>114</v>
       </c>
       <c r="J2">
         <v>10</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="L2">
         <v>0</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="N2">
         <v>0</v>
@@ -1619,43 +1607,43 @@
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D3" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="F3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G3" s="2" t="s">
+      <c r="I3" s="2" t="s">
         <v>119</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>121</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="L3">
         <v>10</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="N3">
         <v>0</v>
@@ -1681,43 +1669,43 @@
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>124</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>126</v>
       </c>
       <c r="J4">
         <v>10</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="L4">
         <v>0</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="N4">
         <v>0</v>
@@ -1743,43 +1731,43 @@
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
       <c r="C5" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="F5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="I5" s="2" t="s">
         <v>129</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>131</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="L5">
         <v>10</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="N5">
         <v>0</v>
@@ -1805,43 +1793,43 @@
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B6">
         <v>2</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G6" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="I6" s="2" t="s">
         <v>112</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>114</v>
       </c>
       <c r="J6">
         <v>10</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="L6">
         <v>0</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="N6">
         <v>0</v>
@@ -1867,43 +1855,43 @@
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E7" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="I7" s="2" t="s">
         <v>135</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>137</v>
       </c>
       <c r="J7">
         <v>10</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="L7">
         <v>0</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="N7">
         <v>0</v>
@@ -1929,43 +1917,43 @@
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B8">
         <v>1</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="I8" s="2" t="s">
         <v>139</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>141</v>
       </c>
       <c r="J8">
         <v>10</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="L8">
         <v>0</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="N8">
         <v>0</v>
@@ -1991,43 +1979,43 @@
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D9" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="I9" s="2" t="s">
         <v>143</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>145</v>
       </c>
       <c r="J9">
         <v>0</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="L9">
         <v>10</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="N9">
         <v>0</v>
@@ -2053,43 +2041,43 @@
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B10">
         <v>2</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="J10">
         <v>10</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="L10">
         <v>0</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="N10">
         <v>0</v>
@@ -3442,321 +3430,321 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>149</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>152</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>154</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>155</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>157</v>
-      </c>
       <c r="C6" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>154</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>154</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>154</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B19" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>154</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>154</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B26" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>154</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Improve Inroads MVP template download and trim list import UI.
Add a download menu with or without media, write on-screen defaults into the workbook, drop Q4 from the Lesson sheet, and remove the list-page zip card.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/inroads-mvp-import-template/lesson.xlsx
+++ b/public/inroads-mvp-import-template/lesson.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="813" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="811" uniqueCount="162">
   <si>
     <t>key</t>
   </si>
@@ -107,9 +107,6 @@
   </si>
   <si>
     <t>Q3</t>
-  </si>
-  <si>
-    <t>Q4</t>
   </si>
   <si>
     <t>Observation</t>
@@ -892,7 +889,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1097,14 +1094,6 @@
       </c>
       <c r="B25" s="2" t="s">
         <v>33</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>34</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -1126,332 +1115,332 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" t="s">
         <v>38</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>41</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>45</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>49</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>51</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>53</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B10" t="s">
+        <v>54</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>55</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B11" t="s">
+        <v>56</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>57</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B12" t="s">
+        <v>58</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B13" t="s">
+        <v>60</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>61</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B14" t="s">
+        <v>62</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>63</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B15" t="s">
+        <v>64</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B16" t="s">
+        <v>66</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>67</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B17" t="s">
+        <v>68</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>69</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B18" t="s">
+        <v>70</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>71</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B19" t="s">
+        <v>72</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>73</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B20" t="s">
+        <v>74</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>76</v>
+      </c>
+      <c r="B21" t="s">
+        <v>38</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>77</v>
-      </c>
-      <c r="B21" t="s">
-        <v>39</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B22" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B23" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B24" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B25" t="s">
+        <v>80</v>
+      </c>
+      <c r="C25" t="s">
         <v>81</v>
-      </c>
-      <c r="C25" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>82</v>
+      </c>
+      <c r="B26" t="s">
+        <v>38</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>83</v>
-      </c>
-      <c r="B26" t="s">
-        <v>39</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B27" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B28" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B29" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B30" t="s">
+        <v>80</v>
+      </c>
+      <c r="C30" t="s">
         <v>81</v>
-      </c>
-      <c r="C30" t="s">
-        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -1483,105 +1472,105 @@
   <sheetData>
     <row r="1" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>105</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>112</v>
       </c>
       <c r="J2">
         <v>10</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="L2">
         <v>0</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="N2">
         <v>0</v>
@@ -1607,43 +1596,43 @@
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D3" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="F3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="I3" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>119</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="L3">
         <v>10</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="N3">
         <v>0</v>
@@ -1669,43 +1658,43 @@
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>123</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>124</v>
       </c>
       <c r="J4">
         <v>10</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L4">
         <v>0</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="N4">
         <v>0</v>
@@ -1731,43 +1720,43 @@
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
       <c r="C5" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="I5" s="2" t="s">
         <v>128</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>129</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="L5">
         <v>10</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="N5">
         <v>0</v>
@@ -1793,43 +1782,43 @@
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B6">
         <v>2</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D6" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>133</v>
-      </c>
       <c r="F6" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G6" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="H6" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="I6" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>112</v>
       </c>
       <c r="J6">
         <v>10</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L6">
         <v>0</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="N6">
         <v>0</v>
@@ -1855,43 +1844,43 @@
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D7" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="I7" s="2" t="s">
         <v>134</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>135</v>
       </c>
       <c r="J7">
         <v>10</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="L7">
         <v>0</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="N7">
         <v>0</v>
@@ -1917,43 +1906,43 @@
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B8">
         <v>1</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="F8" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="I8" s="2" t="s">
         <v>138</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>139</v>
       </c>
       <c r="J8">
         <v>10</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="L8">
         <v>0</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="N8">
         <v>0</v>
@@ -1979,43 +1968,43 @@
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D9" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="F9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="I9" s="2" t="s">
         <v>142</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>143</v>
       </c>
       <c r="J9">
         <v>0</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="L9">
         <v>10</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="N9">
         <v>0</v>
@@ -2041,43 +2030,43 @@
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B10">
         <v>2</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G10" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="H10" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="H10" s="2" t="s">
-        <v>111</v>
-      </c>
       <c r="I10" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J10">
         <v>10</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L10">
         <v>0</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="N10">
         <v>0</v>
@@ -3430,65 +3419,65 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>148</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>151</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>153</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>57</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>151</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>154</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>155</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>156</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>10</v>
@@ -3496,43 +3485,43 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>153</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>57</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>151</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>10</v>
@@ -3540,43 +3529,43 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>153</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>57</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>151</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>10</v>
@@ -3584,43 +3573,43 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>153</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>57</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>151</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>10</v>
@@ -3628,43 +3617,43 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B19" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>153</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B20" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>57</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B21" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>151</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>10</v>
@@ -3672,76 +3661,76 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>153</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B24" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>57</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B25" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>151</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B26" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>153</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>57</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B28" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>151</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
Remove the Metadata tab from lesson workbooks.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/inroads-mvp-import-template/lesson.xlsx
+++ b/public/inroads-mvp-import-template/lesson.xlsx
@@ -7,14 +7,13 @@
     <sheet sheetId="1" name="Lesson" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Instructions" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="Questions" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Metadata" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="811" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="724" uniqueCount="146">
   <si>
     <t>key</t>
   </si>
@@ -458,54 +457,6 @@
   </si>
   <si>
     <t>Here is a coaching question for anticipate?</t>
-  </si>
-  <si>
-    <t>Video Folder</t>
-  </si>
-  <si>
-    <t>Metadata Name</t>
-  </si>
-  <si>
-    <t>Metadata text</t>
-  </si>
-  <si>
-    <t>Observe Hazard Scenario</t>
-  </si>
-  <si>
-    <t>Country</t>
-  </si>
-  <si>
-    <t>Canada</t>
-  </si>
-  <si>
-    <t>Vehicle Type</t>
-  </si>
-  <si>
-    <t>Passenger Vehicle</t>
-  </si>
-  <si>
-    <t>Observe Coaching Video</t>
-  </si>
-  <si>
-    <t>Language</t>
-  </si>
-  <si>
-    <t>Process Lesson Video</t>
-  </si>
-  <si>
-    <t>Process Coaching Video</t>
-  </si>
-  <si>
-    <t>Anticipate Lesson Video</t>
-  </si>
-  <si>
-    <t>Anticipate Coaching Video</t>
-  </si>
-  <si>
-    <t>Observe Explanation Image</t>
-  </si>
-  <si>
-    <t>Hazard Summary Audio</t>
   </si>
 </sst>
 </file>
@@ -3405,340 +3356,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C29"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="48" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>149</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>149</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>149</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>154</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>154</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>154</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>154</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>156</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>156</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>156</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>156</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>157</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>157</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>157</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>157</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>158</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>158</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>158</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>158</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>159</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>159</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>159</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>159</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>160</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>160</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>160</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>161</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>161</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-  </sheetData>
-  <sheetProtection sheet="1" insertRows="0" deleteRows="0"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add the Observe Example button label to lesson workbooks so it can be translated.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/inroads-mvp-import-template/lesson.xlsx
+++ b/public/inroads-mvp-import-template/lesson.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="690" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="695" uniqueCount="190">
   <si>
     <t>Screen</t>
   </si>
@@ -70,6 +70,15 @@
     <t xml:space="preserve">You're about to watch a short driving video. 
 The primary hazard could be in front, behind, or to either side. Drag the screen side-to-side to scan the road and mirrors, then tap or click it as soon as you spot it. 
 You'll have a few seconds and three attempts. No replay, so watch closely.</t>
+  </si>
+  <si>
+    <t>Example button</t>
+  </si>
+  <si>
+    <t>Example</t>
+  </si>
+  <si>
+    <t>When an example video is available</t>
   </si>
   <si>
     <t>Observe challenge</t>
@@ -964,7 +973,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E138"/>
+  <dimension ref="A1:E139"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="27" customWidth="1"/>
@@ -1111,41 +1120,41 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" t="s">
         <v>19</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="D9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" t="s">
         <v>21</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E9" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" t="s">
         <v>23</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="D10" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" t="s">
         <v>25</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E10" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B11" t="s">
         <v>27</v>
@@ -1157,63 +1166,63 @@
         <v>28</v>
       </c>
       <c r="E11" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E12" t="s">
         <v>29</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E12" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E13" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B14" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E14" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="B15" t="s">
         <v>36</v>
@@ -1225,32 +1234,32 @@
         <v>37</v>
       </c>
       <c r="E15" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B16" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E16" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B17" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>42</v>
@@ -1264,78 +1273,78 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B18" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B19" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B20" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E20" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B21" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E21" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B22" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>53</v>
@@ -1349,203 +1358,203 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B23" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>13</v>
+        <v>56</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>13</v>
+        <v>56</v>
       </c>
       <c r="E23" t="s">
-        <v>8</v>
+        <v>57</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="B24" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>56</v>
+        <v>13</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>56</v>
+        <v>13</v>
       </c>
       <c r="E24" t="s">
-        <v>57</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B25" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E25" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B26" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>13</v>
+        <v>61</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>13</v>
+        <v>61</v>
       </c>
       <c r="E26" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B27" t="s">
+        <v>12</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E27" t="s">
         <v>60</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="E27" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B28" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E28" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B29" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E29" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B30" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E30" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B31" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E31" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B32" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>13</v>
+        <v>71</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>13</v>
+        <v>71</v>
       </c>
       <c r="E32" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="B33" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>71</v>
+        <v>13</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>71</v>
+        <v>13</v>
       </c>
       <c r="E33" t="s">
-        <v>8</v>
+        <v>72</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B34" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E34" t="s">
         <v>8</v>
@@ -1553,16 +1562,16 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B35" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>13</v>
+        <v>75</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>13</v>
+        <v>75</v>
       </c>
       <c r="E35" t="s">
         <v>8</v>
@@ -1573,13 +1582,13 @@
         <v>73</v>
       </c>
       <c r="B36" t="s">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>74</v>
+        <v>13</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>74</v>
+        <v>13</v>
       </c>
       <c r="E36" t="s">
         <v>8</v>
@@ -1587,16 +1596,16 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B37" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E37" t="s">
         <v>8</v>
@@ -1604,16 +1613,16 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B38" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E38" t="s">
         <v>8</v>
@@ -1621,16 +1630,16 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B39" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E39" t="s">
         <v>8</v>
@@ -1638,67 +1647,67 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B40" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E40" t="s">
-        <v>69</v>
+        <v>8</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B41" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>13</v>
+        <v>83</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>13</v>
+        <v>83</v>
       </c>
       <c r="E41" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="B42" t="s">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>82</v>
+        <v>13</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>82</v>
+        <v>13</v>
       </c>
       <c r="E42" t="s">
-        <v>8</v>
+        <v>72</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B43" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E43" t="s">
         <v>8</v>
@@ -1706,16 +1715,16 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B44" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E44" t="s">
         <v>8</v>
@@ -1723,16 +1732,16 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B45" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>65</v>
+        <v>87</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>65</v>
+        <v>87</v>
       </c>
       <c r="E45" t="s">
         <v>8</v>
@@ -1740,67 +1749,67 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B46" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="E46" t="s">
-        <v>69</v>
+        <v>8</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B47" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>13</v>
+        <v>88</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>13</v>
+        <v>88</v>
       </c>
       <c r="E47" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B48" t="s">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>87</v>
+        <v>13</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>87</v>
+        <v>13</v>
       </c>
       <c r="E48" t="s">
-        <v>8</v>
+        <v>72</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B49" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E49" t="s">
         <v>8</v>
@@ -1808,16 +1817,16 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B50" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E50" t="s">
         <v>8</v>
@@ -1825,16 +1834,16 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B51" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E51" t="s">
         <v>8</v>
@@ -1842,237 +1851,237 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B52" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E52" t="s">
-        <v>69</v>
+        <v>8</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B53" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E53" t="s">
-        <v>93</v>
+        <v>72</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B54" t="s">
         <v>12</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>13</v>
+        <v>95</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>13</v>
+        <v>95</v>
       </c>
       <c r="E54" t="s">
-        <v>69</v>
+        <v>96</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="B55" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>95</v>
+        <v>13</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>95</v>
+        <v>13</v>
       </c>
       <c r="E55" t="s">
-        <v>96</v>
+        <v>72</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B56" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E56" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B57" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>13</v>
+        <v>100</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>13</v>
+        <v>100</v>
       </c>
       <c r="E57" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B58" t="s">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="C58" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E58" t="s">
         <v>99</v>
-      </c>
-      <c r="D58" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="E58" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B59" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>63</v>
+        <v>102</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>63</v>
+        <v>102</v>
       </c>
       <c r="E59" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B60" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E60" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B61" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="E61" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B62" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>101</v>
+        <v>70</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>101</v>
+        <v>70</v>
       </c>
       <c r="E62" t="s">
-        <v>69</v>
+        <v>103</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B63" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>13</v>
+        <v>104</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>13</v>
+        <v>104</v>
       </c>
       <c r="E63" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B64" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>103</v>
+        <v>13</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>103</v>
+        <v>13</v>
       </c>
       <c r="E64" t="s">
-        <v>8</v>
+        <v>72</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B65" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E65" t="s">
         <v>8</v>
@@ -2080,16 +2089,16 @@
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B66" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>13</v>
+        <v>107</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>13</v>
+        <v>107</v>
       </c>
       <c r="E66" t="s">
         <v>8</v>
@@ -2100,13 +2109,13 @@
         <v>105</v>
       </c>
       <c r="B67" t="s">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>106</v>
+        <v>13</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>106</v>
+        <v>13</v>
       </c>
       <c r="E67" t="s">
         <v>8</v>
@@ -2114,16 +2123,16 @@
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B68" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E68" t="s">
         <v>8</v>
@@ -2131,16 +2140,16 @@
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B69" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E69" t="s">
         <v>8</v>
@@ -2148,16 +2157,16 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B70" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E70" t="s">
         <v>8</v>
@@ -2165,67 +2174,67 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B71" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="E71" t="s">
-        <v>69</v>
+        <v>8</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B72" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>13</v>
+        <v>104</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>13</v>
+        <v>104</v>
       </c>
       <c r="E72" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B73" t="s">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>110</v>
+        <v>13</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>110</v>
+        <v>13</v>
       </c>
       <c r="E73" t="s">
-        <v>8</v>
+        <v>72</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B74" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E74" t="s">
         <v>8</v>
@@ -2233,16 +2242,16 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B75" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E75" t="s">
         <v>8</v>
@@ -2250,16 +2259,16 @@
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B76" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="E76" t="s">
         <v>8</v>
@@ -2267,67 +2276,67 @@
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B77" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E77" t="s">
-        <v>69</v>
+        <v>8</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B78" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>13</v>
+        <v>116</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>13</v>
+        <v>116</v>
       </c>
       <c r="E78" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B79" t="s">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>115</v>
+        <v>13</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>115</v>
+        <v>13</v>
       </c>
       <c r="E79" t="s">
-        <v>8</v>
+        <v>72</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B80" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E80" t="s">
         <v>8</v>
@@ -2335,16 +2344,16 @@
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B81" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E81" t="s">
         <v>8</v>
@@ -2352,16 +2361,16 @@
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B82" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E82" t="s">
         <v>8</v>
@@ -2369,206 +2378,206 @@
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B83" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E83" t="s">
-        <v>69</v>
+        <v>8</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B84" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>92</v>
+        <v>122</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>92</v>
+        <v>122</v>
       </c>
       <c r="E84" t="s">
-        <v>93</v>
+        <v>72</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B85" t="s">
         <v>12</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>13</v>
+        <v>95</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>13</v>
+        <v>95</v>
       </c>
       <c r="E85" t="s">
-        <v>69</v>
+        <v>96</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B86" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>121</v>
+        <v>13</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>121</v>
+        <v>13</v>
       </c>
       <c r="E86" t="s">
-        <v>122</v>
+        <v>72</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B87" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E87" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B88" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>13</v>
+        <v>126</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>13</v>
+        <v>126</v>
       </c>
       <c r="E88" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B89" t="s">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="C89" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D89" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E89" t="s">
         <v>125</v>
-      </c>
-      <c r="D89" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="E89" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B90" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>83</v>
+        <v>128</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>83</v>
+        <v>128</v>
       </c>
       <c r="E90" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B91" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E91" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B92" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="E92" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B93" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>113</v>
+        <v>87</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>113</v>
+        <v>87</v>
       </c>
       <c r="E93" t="s">
-        <v>69</v>
+        <v>129</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B94" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>13</v>
+        <v>116</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>13</v>
+        <v>116</v>
       </c>
       <c r="E94" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
@@ -2576,58 +2585,58 @@
         <v>127</v>
       </c>
       <c r="B95" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D95" s="1" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E95" t="s">
-        <v>8</v>
+        <v>72</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B96" t="s">
-        <v>128</v>
+        <v>5</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>129</v>
+        <v>9</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>129</v>
+        <v>9</v>
       </c>
       <c r="E96" t="s">
-        <v>130</v>
+        <v>8</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B97" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D97" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E97" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B98" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C98" s="1" t="s">
         <v>134</v>
@@ -2636,21 +2645,21 @@
         <v>134</v>
       </c>
       <c r="E98" t="s">
-        <v>8</v>
+        <v>135</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B99" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D99" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E99" t="s">
         <v>8</v>
@@ -2658,16 +2667,16 @@
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B100" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>71</v>
+        <v>139</v>
       </c>
       <c r="D100" s="1" t="s">
-        <v>71</v>
+        <v>139</v>
       </c>
       <c r="E100" t="s">
         <v>8</v>
@@ -2675,16 +2684,16 @@
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B101" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>137</v>
+        <v>74</v>
       </c>
       <c r="D101" s="1" t="s">
-        <v>137</v>
+        <v>74</v>
       </c>
       <c r="E101" t="s">
         <v>8</v>
@@ -2692,24 +2701,24 @@
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B102" t="s">
         <v>138</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D102" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E102" t="s">
-        <v>140</v>
+        <v>8</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B103" t="s">
         <v>141</v>
@@ -2721,123 +2730,123 @@
         <v>142</v>
       </c>
       <c r="E103" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B104" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D104" s="1" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="E104" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B105" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D105" s="1" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E105" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B106" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D106" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E106" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B107" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D107" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E107" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B108" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D108" s="1" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="E108" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B109" t="s">
+        <v>144</v>
+      </c>
+      <c r="C109" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="D109" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="E109" t="s">
         <v>150</v>
-      </c>
-      <c r="C109" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="D109" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="E109" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B110" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D110" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E110" t="s">
         <v>8</v>
@@ -2845,16 +2854,16 @@
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B111" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D111" s="1" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E111" t="s">
         <v>8</v>
@@ -2862,16 +2871,16 @@
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B112" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D112" s="1" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E112" t="s">
         <v>8</v>
@@ -2879,16 +2888,16 @@
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B113" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D113" s="1" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E113" t="s">
         <v>8</v>
@@ -2896,16 +2905,16 @@
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B114" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D114" s="1" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E114" t="s">
         <v>8</v>
@@ -2913,16 +2922,16 @@
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B115" t="s">
-        <v>12</v>
+        <v>153</v>
       </c>
       <c r="C115" s="1" t="s">
-        <v>13</v>
+        <v>159</v>
       </c>
       <c r="D115" s="1" t="s">
-        <v>13</v>
+        <v>159</v>
       </c>
       <c r="E115" t="s">
         <v>8</v>
@@ -2930,44 +2939,44 @@
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>157</v>
+        <v>130</v>
       </c>
       <c r="B116" t="s">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="C116" s="1" t="s">
-        <v>157</v>
+        <v>13</v>
       </c>
       <c r="D116" s="1" t="s">
-        <v>157</v>
+        <v>13</v>
       </c>
       <c r="E116" t="s">
-        <v>158</v>
+        <v>8</v>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B117" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D117" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E117" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B118" t="s">
-        <v>161</v>
+        <v>39</v>
       </c>
       <c r="C118" s="1" t="s">
         <v>162</v>
@@ -2976,351 +2985,368 @@
         <v>162</v>
       </c>
       <c r="E118" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B119" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="C119" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="D119" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="E119" t="s">
         <v>163</v>
-      </c>
-      <c r="D119" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="E119" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B120" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D120" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="E120" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B121" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D121" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="E121" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B122" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="C122" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D122" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="E122" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B123" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="C123" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D123" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="E123" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B124" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D124" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E124" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B125" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D125" s="1" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="E125" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B126" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D126" s="1" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E126" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B127" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D127" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E127" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B128" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D128" s="1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E128" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B129" t="s">
-        <v>36</v>
+        <v>175</v>
       </c>
       <c r="C129" s="1" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="D129" s="1" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="E129" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B130" t="s">
-        <v>176</v>
+        <v>39</v>
       </c>
       <c r="C130" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D130" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E130" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B131" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C131" s="1" t="s">
-        <v>155</v>
+        <v>180</v>
       </c>
       <c r="D131" s="1" t="s">
-        <v>155</v>
+        <v>180</v>
       </c>
       <c r="E131" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B132" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C132" s="1" t="s">
-        <v>180</v>
+        <v>158</v>
       </c>
       <c r="D132" s="1" t="s">
-        <v>180</v>
+        <v>158</v>
       </c>
       <c r="E132" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B133" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="D133" s="1" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="E133" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B134" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C134" s="1" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D134" s="1" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="E134" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B135" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="C135" s="1" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D135" s="1" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="E135" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B136" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C136" s="1" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D136" s="1" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E136" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B137" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="C137" s="1" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="D137" s="1" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="E137" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B138" t="s">
+        <v>181</v>
+      </c>
+      <c r="C138" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="D138" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="E138" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
+        <v>160</v>
+      </c>
+      <c r="B139" t="s">
         <v>12</v>
       </c>
-      <c r="C138" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="D138" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="E138" t="s">
-        <v>160</v>
+      <c r="C139" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="D139" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="E139" t="s">
+        <v>163</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>